<commit_message>
Edited other.txt and README.md + Fixed formatting for stats & updated wikipedia checker w/ GEMINI
</commit_message>
<xml_diff>
--- a/books_input.xlsx
+++ b/books_input.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="41">
   <si>
     <t>To Kill a Mockingbird</t>
   </si>
@@ -103,23 +103,44 @@
     <t>The Lord of the Rings</t>
   </si>
   <si>
-    <t>FAKE BOOK TITLE 123</t>
-  </si>
-  <si>
-    <t>불편한 편의점</t>
-  </si>
-  <si>
-    <t>김호연</t>
-  </si>
-  <si>
-    <t>힐링 소설</t>
+    <t>Cien años de soledad</t>
+  </si>
+  <si>
+    <t>Gabriel García Márquez</t>
+  </si>
+  <si>
+    <t>Realismo mágico</t>
+  </si>
+  <si>
+    <t>One Hundred Years of Solitude</t>
+  </si>
+  <si>
+    <t>Magical Realism</t>
+  </si>
+  <si>
+    <t>채식주의자</t>
+  </si>
+  <si>
+    <t>한강</t>
+  </si>
+  <si>
+    <t>문학</t>
+  </si>
+  <si>
+    <t>blahl balba hla FAKE</t>
+  </si>
+  <si>
+    <t>bla hb bl31414</t>
+  </si>
+  <si>
+    <t>&amp;#(*@($#df</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -134,11 +155,6 @@
       <color theme="1"/>
       <name val="Arial"/>
     </font>
-    <font>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -149,31 +165,31 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFF6F8F9"/>
+        <bgColor rgb="FFF6F8F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF6F8F9"/>
-        <bgColor rgb="FFF6F8F9"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="8">
+  <borders count="3">
     <border/>
     <border>
       <left style="thin">
-        <color rgb="FF284E3F"/>
+        <color rgb="FFF6F8F9"/>
       </left>
       <right style="thin">
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFF6F8F9"/>
       </right>
       <top style="thin">
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFF6F8F9"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFF6F8F9"/>
       </bottom>
     </border>
     <border>
@@ -190,124 +206,29 @@
         <color rgb="FFFFFFFF"/>
       </bottom>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFFFFFFF"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF284E3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFFFFFFF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFFFFFFF"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF284E3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFF6F8F9"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFF6F8F9"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFF6F8F9"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFF6F8F9"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFF6F8F9"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFF6F8F9"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFF6F8F9"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFF6F8F9"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF284E3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFF6F8F9"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFF6F8F9"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF284E3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFF6F8F9"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFF6F8F9"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF284E3F"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="6">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="right" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="2" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="3" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="right" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="5" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="5" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="6" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="2" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="3" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="5" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="6" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="2" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="7" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="right" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf borderId="2" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -359,7 +280,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A1:D14" displayName="Table_1" name="Table_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A1:D22" displayName="Table_1" name="Table_1" id="1">
   <tableColumns count="4">
     <tableColumn name="Column1" id="1"/>
     <tableColumn name="Column2" id="2"/>
@@ -580,215 +501,267 @@
       <c r="A1" s="1">
         <v>1.0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4">
+      <c r="A2" s="2">
         <v>2.0</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>3.0</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4">
+      <c r="A4" s="2">
         <v>4.0</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="12"/>
+      <c r="E4" s="3"/>
     </row>
     <row r="5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>5.0</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4">
+      <c r="A6" s="2">
         <v>6.0</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="12"/>
+      <c r="E6" s="3"/>
     </row>
     <row r="7">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>7.0</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="2" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4">
+      <c r="A8" s="2">
         <v>8.0</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="12"/>
+      <c r="E8" s="3"/>
     </row>
     <row r="9">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>9.0</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="2" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4">
+      <c r="A10" s="2">
         <v>10.0</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E10" s="12"/>
+      <c r="E10" s="3"/>
     </row>
     <row r="11">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>11.0</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="D11" s="9" t="s">
+      <c r="C11" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4">
+      <c r="A12" s="2">
         <v>12.0</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="11" t="s">
+      <c r="D12" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="E12" s="12"/>
+      <c r="E12" s="3"/>
     </row>
     <row r="13">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>13.0</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C13" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="D13" s="9" t="s">
-        <v>28</v>
+      <c r="C13" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="13">
+      <c r="A14" s="2">
         <v>14.0</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="E14" s="12"/>
+      <c r="D14" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E14" s="3"/>
     </row>
     <row r="15">
-      <c r="A15" s="14"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
+      <c r="A15" s="2">
+        <v>15.0</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="14"/>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
+      <c r="A16" s="4">
+        <v>16.0</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="5"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="5"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="5"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Added txt files + Changed whole structure of wiki book checker file. Explained in Note.txt
</commit_message>
<xml_diff>
--- a/books_input.xlsx
+++ b/books_input.xlsx
@@ -11,7 +11,16 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="36">
+  <si>
+    <t>The Haunting of Hill House</t>
+  </si>
+  <si>
+    <t>Shirley Jackson</t>
+  </si>
+  <si>
+    <t>Psychological horror</t>
+  </si>
   <si>
     <t>To Kill a Mockingbird</t>
   </si>
@@ -31,109 +40,85 @@
     <t>FAKE</t>
   </si>
   <si>
-    <t>The Great Gatsby</t>
-  </si>
-  <si>
-    <t>F. Scott Fitzgerald</t>
-  </si>
-  <si>
-    <t>Pride and Prejudice</t>
-  </si>
-  <si>
-    <t>Jane Austen</t>
-  </si>
-  <si>
-    <t>Romance</t>
-  </si>
-  <si>
-    <t>The Catcher in the Rye</t>
-  </si>
-  <si>
-    <t>J.D. Salinger</t>
-  </si>
-  <si>
-    <t>Brave New World</t>
-  </si>
-  <si>
-    <t>Aldous Huxley</t>
-  </si>
-  <si>
-    <t>Dystopian</t>
-  </si>
-  <si>
-    <t>The Hobbit</t>
+    <t>One Hundred Years of Solitude</t>
+  </si>
+  <si>
+    <t>Gabriel García Márquez</t>
+  </si>
+  <si>
+    <t>Magical Realism</t>
+  </si>
+  <si>
+    <t>战争与和平</t>
+  </si>
+  <si>
+    <t>列夫·托尔斯泰</t>
+  </si>
+  <si>
+    <t>小说 / 历史小说</t>
+  </si>
+  <si>
+    <t>THE LORD OF THE RINGS</t>
   </si>
   <si>
     <t>J.R.R. Tolkien</t>
   </si>
   <si>
+    <t>FANTASY</t>
+  </si>
+  <si>
+    <t>Преступление и наказание</t>
+  </si>
+  <si>
+    <t>Фёдор Михайлович Достоевский</t>
+  </si>
+  <si>
+    <t>философский роман</t>
+  </si>
+  <si>
+    <t>The HObBit</t>
+  </si>
+  <si>
+    <t>FantASY</t>
+  </si>
+  <si>
+    <t>채식주의자</t>
+  </si>
+  <si>
+    <t>한강</t>
+  </si>
+  <si>
+    <t>문학</t>
+  </si>
+  <si>
+    <t>Gone with the Wind</t>
+  </si>
+  <si>
+    <t>Margaret Mitchell</t>
+  </si>
+  <si>
+    <t>Historical Fiction</t>
+  </si>
+  <si>
+    <t>blahl balba hla FAKE</t>
+  </si>
+  <si>
+    <t>bla hb bl31414</t>
+  </si>
+  <si>
+    <t>&amp;#(*@($#df</t>
+  </si>
+  <si>
+    <t>The Lord of the Rings</t>
+  </si>
+  <si>
     <t>Fantasy</t>
   </si>
   <si>
-    <t>Harry Potter and the Philosopher's Stone</t>
-  </si>
-  <si>
-    <t>J.K. Rowling</t>
-  </si>
-  <si>
-    <t>The Da Vinci Code</t>
-  </si>
-  <si>
-    <t>Dan Brown</t>
-  </si>
-  <si>
-    <t>Mystery</t>
-  </si>
-  <si>
-    <t>Gone with the Wind</t>
-  </si>
-  <si>
-    <t>Margaret Mitchell</t>
-  </si>
-  <si>
-    <t>Historical Fiction</t>
-  </si>
-  <si>
-    <t>FAKE BOOK TITLE XYZ123</t>
-  </si>
-  <si>
-    <t>Unknown</t>
-  </si>
-  <si>
-    <t>The Lord of the Rings</t>
-  </si>
-  <si>
     <t>Cien años de soledad</t>
   </si>
   <si>
-    <t>Gabriel García Márquez</t>
-  </si>
-  <si>
     <t>Realismo mágico</t>
-  </si>
-  <si>
-    <t>One Hundred Years of Solitude</t>
-  </si>
-  <si>
-    <t>Magical Realism</t>
-  </si>
-  <si>
-    <t>채식주의자</t>
-  </si>
-  <si>
-    <t>한강</t>
-  </si>
-  <si>
-    <t>문학</t>
-  </si>
-  <si>
-    <t>blahl balba hla FAKE</t>
-  </si>
-  <si>
-    <t>bla hb bl31414</t>
-  </si>
-  <si>
-    <t>&amp;#(*@($#df</t>
   </si>
 </sst>
 </file>
@@ -210,7 +195,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -218,16 +203,28 @@
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="2" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="2" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
     <xf borderId="2" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="2" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -262,8 +259,12 @@
       <border/>
     </dxf>
   </dxfs>
-  <tableStyles count="1">
+  <tableStyles count="2">
     <tableStyle count="2" pivot="0" name="Books to Verify-style">
+      <tableStyleElement dxfId="1" type="firstRowStripe"/>
+      <tableStyleElement dxfId="2" type="secondRowStripe"/>
+    </tableStyle>
+    <tableStyle count="2" pivot="0" name="Books to Verify-style 2">
       <tableStyleElement dxfId="1" type="firstRowStripe"/>
       <tableStyleElement dxfId="2" type="secondRowStripe"/>
     </tableStyle>
@@ -280,7 +281,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A1:D22" displayName="Table_1" name="Table_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A1:D25" displayName="Table_1" name="Table_1" id="1">
   <tableColumns count="4">
     <tableColumn name="Column1" id="1"/>
     <tableColumn name="Column2" id="2"/>
@@ -288,6 +289,18 @@
     <tableColumn name="Column4" id="4"/>
   </tableColumns>
   <tableStyleInfo name="Books to Verify-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="H9:K27" displayName="Table_2" name="Table_2" id="2">
+  <tableColumns count="4">
+    <tableColumn name="Column1" id="1"/>
+    <tableColumn name="Column2" id="2"/>
+    <tableColumn name="Column3" id="3"/>
+    <tableColumn name="Column4" id="4"/>
+  </tableColumns>
+  <tableStyleInfo name="Books to Verify-style 2" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
 </table>
 </file>
 
@@ -501,27 +514,27 @@
       <c r="A1" s="1">
         <v>1.0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="3">
         <v>2.0</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -529,43 +542,43 @@
       <c r="A3" s="2">
         <v>3.0</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>2</v>
+      <c r="D3" s="3" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2">
+      <c r="A4" s="3">
         <v>4.0</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="3"/>
+      <c r="D4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="4"/>
     </row>
     <row r="5">
       <c r="A5" s="2">
         <v>5.0</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6">
@@ -573,200 +586,300 @@
         <v>6.0</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" s="3"/>
+        <v>17</v>
+      </c>
+      <c r="E6" s="4"/>
     </row>
     <row r="7">
       <c r="A7" s="2">
         <v>7.0</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5">
+        <v>8.0</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2">
-        <v>8.0</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="D8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E8" s="3"/>
+        <v>22</v>
+      </c>
+      <c r="E8" s="4"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
     </row>
     <row r="9">
       <c r="A9" s="2">
         <v>9.0</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>23</v>
       </c>
+      <c r="C9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
     </row>
     <row r="10">
       <c r="A10" s="2">
         <v>10.0</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D10" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E10" s="3"/>
+      <c r="C10" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" s="4"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
     </row>
     <row r="11">
       <c r="A11" s="2">
         <v>11.0</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>5</v>
+        <v>29</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>30</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>28</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
     </row>
     <row r="12">
       <c r="A12" s="2">
         <v>12.0</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E12" s="3"/>
+      <c r="B12" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E12" s="4"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="6"/>
+      <c r="J12" s="6"/>
+      <c r="K12" s="6"/>
     </row>
     <row r="13">
       <c r="A13" s="2">
         <v>13.0</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>32</v>
-      </c>
+      <c r="B13" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G13" s="3"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="3"/>
     </row>
     <row r="14">
       <c r="A14" s="2">
         <v>14.0</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E14" s="3"/>
+      <c r="B14" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" s="4"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="2"/>
     </row>
     <row r="15">
-      <c r="A15" s="2">
-        <v>15.0</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>37</v>
-      </c>
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="K15" s="3"/>
     </row>
     <row r="16">
-      <c r="A16" s="4">
-        <v>16.0</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>40</v>
-      </c>
+      <c r="A16" s="3"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+      <c r="J16" s="3"/>
+      <c r="K16" s="3"/>
     </row>
     <row r="17">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
+      <c r="A17" s="3"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
       <c r="D17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="6"/>
+      <c r="I17" s="6"/>
+      <c r="J17" s="6"/>
+      <c r="K17" s="2"/>
     </row>
     <row r="18">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
+      <c r="A18" s="3"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
       <c r="D18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
+      <c r="J18" s="3"/>
+      <c r="K18" s="3"/>
     </row>
     <row r="19">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
+      <c r="A19" s="3"/>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
       <c r="D19" s="2"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
+      <c r="K19" s="3"/>
     </row>
     <row r="20">
-      <c r="A20" s="2"/>
+      <c r="A20" s="3"/>
       <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="5"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="2"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+      <c r="J20" s="3"/>
+      <c r="K20" s="3"/>
     </row>
     <row r="21">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="5"/>
+      <c r="A21" s="3"/>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="2"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="K21" s="3"/>
     </row>
     <row r="22">
-      <c r="A22" s="2"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="5"/>
+      <c r="A22" s="3"/>
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="7"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="8"/>
+      <c r="B23" s="3"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="7"/>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
+      <c r="J23" s="2"/>
+      <c r="K23" s="3"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="8"/>
+      <c r="B24" s="3"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="7"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+      <c r="K24" s="2"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="8"/>
+      <c r="B25" s="3"/>
+      <c r="C25" s="8"/>
+      <c r="D25" s="7"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+      <c r="K25" s="9"/>
+    </row>
+    <row r="26">
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+      <c r="J26" s="3"/>
+      <c r="K26" s="9"/>
+    </row>
+    <row r="27">
+      <c r="H27" s="2"/>
+      <c r="I27" s="2"/>
+      <c r="J27" s="3"/>
+      <c r="K27" s="9"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>
-  <tableParts count="1">
-    <tablePart r:id="rId3"/>
+  <tableParts count="2">
+    <tablePart r:id="rId4"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>